<commit_message>
Add best/worst hybrid Holt-Winters scenario sheets
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D73U26FQnMJ6VM9LfvsWf3
</commit_message>
<xml_diff>
--- a/توقع_هولت_وينترز_الهجين_2026.xlsx
+++ b/توقع_هولت_وينترز_الهجين_2026.xlsx
@@ -8,9 +8,11 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الملخص" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="العوامل والدفعات" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="النموذج والاختبار" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="السلسلة الشهرية" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الأفضل" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الأسوأ" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="العوامل والدفعات" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="النموذج والاختبار" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="السلسلة الشهرية" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1063,6 +1065,1678 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:Y11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="13" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="13" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="25" max="25"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>الأفضل: إقفال 2026 بنموذج هولت-وينترز الهجين حسب التبويب (بدون الضريبة)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="44" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>الأفضل = الحد الأعلى لنطاق ثقة 80% لنموذج هولت-وينترز × العوامل الخارجية + الدفعات الاستثنائية المعروفة (تأجير المرافق 441م في نوفمبر)، وأكتوبر لا يقل عن المحصل حتى تاريخه. العوامل والدفعات تُعدَّل من ورقة "العوامل والدفعات".</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>التبويب</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>التراكمي يناير–سبتمبر (فعلي)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n"/>
+      <c r="D4" s="3" t="n"/>
+      <c r="E4" s="3" t="n"/>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>أكتوبر</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="n"/>
+      <c r="H4" s="3" t="n"/>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>نوفمبر</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="n"/>
+      <c r="L4" s="3" t="n"/>
+      <c r="M4" s="3" t="n"/>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>ديسمبر</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="n"/>
+      <c r="P4" s="3" t="n"/>
+      <c r="Q4" s="3" t="n"/>
+      <c r="R4" s="3" t="inlineStr">
+        <is>
+          <t>أكتوبر–ديسمبر</t>
+        </is>
+      </c>
+      <c r="S4" s="3" t="n"/>
+      <c r="T4" s="3" t="n"/>
+      <c r="U4" s="3" t="n"/>
+      <c r="V4" s="3" t="inlineStr">
+        <is>
+          <t>إجمالي السنة 2026</t>
+        </is>
+      </c>
+      <c r="W4" s="3" t="n"/>
+      <c r="X4" s="3" t="n"/>
+      <c r="Y4" s="3" t="n"/>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>المستهدف</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>المحصل / المتوقع</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>الفرق عن المستهدف</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>% من المستهدف</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>المستهدف</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>المحصل / المتوقع</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>الفرق عن المستهدف</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>% من المستهدف</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>المستهدف</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>المحصل / المتوقع</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>الفرق عن المستهدف</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>% من المستهدف</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>المستهدف</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="inlineStr">
+        <is>
+          <t>المحصل / المتوقع</t>
+        </is>
+      </c>
+      <c r="P5" s="3" t="inlineStr">
+        <is>
+          <t>الفرق عن المستهدف</t>
+        </is>
+      </c>
+      <c r="Q5" s="3" t="inlineStr">
+        <is>
+          <t>% من المستهدف</t>
+        </is>
+      </c>
+      <c r="R5" s="3" t="inlineStr">
+        <is>
+          <t>المستهدف</t>
+        </is>
+      </c>
+      <c r="S5" s="3" t="inlineStr">
+        <is>
+          <t>المحصل / المتوقع</t>
+        </is>
+      </c>
+      <c r="T5" s="3" t="inlineStr">
+        <is>
+          <t>الفرق عن المستهدف</t>
+        </is>
+      </c>
+      <c r="U5" s="3" t="inlineStr">
+        <is>
+          <t>% من المستهدف</t>
+        </is>
+      </c>
+      <c r="V5" s="3" t="inlineStr">
+        <is>
+          <t>المستهدف</t>
+        </is>
+      </c>
+      <c r="W5" s="3" t="inlineStr">
+        <is>
+          <t>المحصل / المتوقع</t>
+        </is>
+      </c>
+      <c r="X5" s="3" t="inlineStr">
+        <is>
+          <t>الفرق عن المستهدف</t>
+        </is>
+      </c>
+      <c r="Y5" s="3" t="inlineStr">
+        <is>
+          <t>% من المستهدف</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>1038815836.09</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>1052146902.93</v>
+      </c>
+      <c r="D6" s="5">
+        <f>C6-B6</f>
+        <v/>
+      </c>
+      <c r="E6" s="7">
+        <f>IF(B6=0,"",C6/B6)</f>
+        <v/>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>229687321.85</v>
+      </c>
+      <c r="G6" s="5">
+        <f>MAX(33361604.91,144950797.79*'العوامل والدفعات'!D5+'العوامل والدفعات'!B14)</f>
+        <v/>
+      </c>
+      <c r="H6" s="5">
+        <f>G6-F6</f>
+        <v/>
+      </c>
+      <c r="I6" s="7">
+        <f>IF(F6=0,"",G6/F6)</f>
+        <v/>
+      </c>
+      <c r="J6" s="5" t="n">
+        <v>495549226.08</v>
+      </c>
+      <c r="K6" s="5">
+        <f>147956964.50*'العوامل والدفعات'!D5+'العوامل والدفعات'!C14</f>
+        <v/>
+      </c>
+      <c r="L6" s="5">
+        <f>K6-J6</f>
+        <v/>
+      </c>
+      <c r="M6" s="7">
+        <f>IF(J6=0,"",K6/J6)</f>
+        <v/>
+      </c>
+      <c r="N6" s="5" t="n">
+        <v>63384343.05999999</v>
+      </c>
+      <c r="O6" s="5">
+        <f>114719567.10*'العوامل والدفعات'!D5+'العوامل والدفعات'!D14</f>
+        <v/>
+      </c>
+      <c r="P6" s="5">
+        <f>O6-N6</f>
+        <v/>
+      </c>
+      <c r="Q6" s="7">
+        <f>IF(N6=0,"",O6/N6)</f>
+        <v/>
+      </c>
+      <c r="R6" s="5">
+        <f>F6+J6+N6</f>
+        <v/>
+      </c>
+      <c r="S6" s="5">
+        <f>G6+K6+O6</f>
+        <v/>
+      </c>
+      <c r="T6" s="5">
+        <f>S6-R6</f>
+        <v/>
+      </c>
+      <c r="U6" s="7">
+        <f>IF(R6=0,"",S6/R6)</f>
+        <v/>
+      </c>
+      <c r="V6" s="5">
+        <f>B6+R6</f>
+        <v/>
+      </c>
+      <c r="W6" s="5">
+        <f>C6+S6</f>
+        <v/>
+      </c>
+      <c r="X6" s="5">
+        <f>W6-V6</f>
+        <v/>
+      </c>
+      <c r="Y6" s="7">
+        <f>IF(V6=0,"",W6/V6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>895660932.61</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>893640140.0200001</v>
+      </c>
+      <c r="D7" s="5">
+        <f>C7-B7</f>
+        <v/>
+      </c>
+      <c r="E7" s="7">
+        <f>IF(B7=0,"",C7/B7)</f>
+        <v/>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>96839259.07000001</v>
+      </c>
+      <c r="G7" s="5">
+        <f>MAX(47001537.91,115689354.46*'العوامل والدفعات'!D6+'العوامل والدفعات'!B15)</f>
+        <v/>
+      </c>
+      <c r="H7" s="5">
+        <f>G7-F7</f>
+        <v/>
+      </c>
+      <c r="I7" s="7">
+        <f>IF(F7=0,"",G7/F7)</f>
+        <v/>
+      </c>
+      <c r="J7" s="5" t="n">
+        <v>73087705.87</v>
+      </c>
+      <c r="K7" s="5">
+        <f>106260512.41*'العوامل والدفعات'!D6+'العوامل والدفعات'!C15</f>
+        <v/>
+      </c>
+      <c r="L7" s="5">
+        <f>K7-J7</f>
+        <v/>
+      </c>
+      <c r="M7" s="7">
+        <f>IF(J7=0,"",K7/J7)</f>
+        <v/>
+      </c>
+      <c r="N7" s="5" t="n">
+        <v>91097976.65000002</v>
+      </c>
+      <c r="O7" s="5">
+        <f>133017083.39*'العوامل والدفعات'!D6+'العوامل والدفعات'!D15</f>
+        <v/>
+      </c>
+      <c r="P7" s="5">
+        <f>O7-N7</f>
+        <v/>
+      </c>
+      <c r="Q7" s="7">
+        <f>IF(N7=0,"",O7/N7)</f>
+        <v/>
+      </c>
+      <c r="R7" s="5">
+        <f>F7+J7+N7</f>
+        <v/>
+      </c>
+      <c r="S7" s="5">
+        <f>G7+K7+O7</f>
+        <v/>
+      </c>
+      <c r="T7" s="5">
+        <f>S7-R7</f>
+        <v/>
+      </c>
+      <c r="U7" s="7">
+        <f>IF(R7=0,"",S7/R7)</f>
+        <v/>
+      </c>
+      <c r="V7" s="5">
+        <f>B7+R7</f>
+        <v/>
+      </c>
+      <c r="W7" s="5">
+        <f>C7+S7</f>
+        <v/>
+      </c>
+      <c r="X7" s="5">
+        <f>W7-V7</f>
+        <v/>
+      </c>
+      <c r="Y7" s="7">
+        <f>IF(V7=0,"",W7/V7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>جزاءات وغرامات</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>426733084.54</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>638994901.72</v>
+      </c>
+      <c r="D8" s="5">
+        <f>C8-B8</f>
+        <v/>
+      </c>
+      <c r="E8" s="7">
+        <f>IF(B8=0,"",C8/B8)</f>
+        <v/>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>50463196.19</v>
+      </c>
+      <c r="G8" s="5">
+        <f>MAX(33304429.00,42016411.89*'العوامل والدفعات'!D7+'العوامل والدفعات'!B16)</f>
+        <v/>
+      </c>
+      <c r="H8" s="5">
+        <f>G8-F8</f>
+        <v/>
+      </c>
+      <c r="I8" s="7">
+        <f>IF(F8=0,"",G8/F8)</f>
+        <v/>
+      </c>
+      <c r="J8" s="5" t="n">
+        <v>39418777.06</v>
+      </c>
+      <c r="K8" s="5">
+        <f>41703469.26*'العوامل والدفعات'!D7+'العوامل والدفعات'!C16</f>
+        <v/>
+      </c>
+      <c r="L8" s="5">
+        <f>K8-J8</f>
+        <v/>
+      </c>
+      <c r="M8" s="7">
+        <f>IF(J8=0,"",K8/J8)</f>
+        <v/>
+      </c>
+      <c r="N8" s="5" t="n">
+        <v>44888053.81</v>
+      </c>
+      <c r="O8" s="5">
+        <f>52585115.13*'العوامل والدفعات'!D7+'العوامل والدفعات'!D16</f>
+        <v/>
+      </c>
+      <c r="P8" s="5">
+        <f>O8-N8</f>
+        <v/>
+      </c>
+      <c r="Q8" s="7">
+        <f>IF(N8=0,"",O8/N8)</f>
+        <v/>
+      </c>
+      <c r="R8" s="5">
+        <f>F8+J8+N8</f>
+        <v/>
+      </c>
+      <c r="S8" s="5">
+        <f>G8+K8+O8</f>
+        <v/>
+      </c>
+      <c r="T8" s="5">
+        <f>S8-R8</f>
+        <v/>
+      </c>
+      <c r="U8" s="7">
+        <f>IF(R8=0,"",S8/R8)</f>
+        <v/>
+      </c>
+      <c r="V8" s="5">
+        <f>B8+R8</f>
+        <v/>
+      </c>
+      <c r="W8" s="5">
+        <f>C8+S8</f>
+        <v/>
+      </c>
+      <c r="X8" s="5">
+        <f>W8-V8</f>
+        <v/>
+      </c>
+      <c r="Y8" s="7">
+        <f>IF(V8=0,"",W8/V8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>التبغ والإيواء</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>308355656.8</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>209094919.82</v>
+      </c>
+      <c r="D9" s="5">
+        <f>C9-B9</f>
+        <v/>
+      </c>
+      <c r="E9" s="7">
+        <f>IF(B9=0,"",C9/B9)</f>
+        <v/>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>34427181.46</v>
+      </c>
+      <c r="G9" s="5">
+        <f>MAX(17460981.18,27618510.21*'العوامل والدفعات'!D8+'العوامل والدفعات'!B17)</f>
+        <v/>
+      </c>
+      <c r="H9" s="5">
+        <f>G9-F9</f>
+        <v/>
+      </c>
+      <c r="I9" s="7">
+        <f>IF(F9=0,"",G9/F9)</f>
+        <v/>
+      </c>
+      <c r="J9" s="5" t="n">
+        <v>26865316.43</v>
+      </c>
+      <c r="K9" s="5">
+        <f>32163408.61*'العوامل والدفعات'!D8+'العوامل والدفعات'!C17</f>
+        <v/>
+      </c>
+      <c r="L9" s="5">
+        <f>K9-J9</f>
+        <v/>
+      </c>
+      <c r="M9" s="7">
+        <f>IF(J9=0,"",K9/J9)</f>
+        <v/>
+      </c>
+      <c r="N9" s="5" t="n">
+        <v>29501207.8</v>
+      </c>
+      <c r="O9" s="5">
+        <f>30473567.23*'العوامل والدفعات'!D8+'العوامل والدفعات'!D17</f>
+        <v/>
+      </c>
+      <c r="P9" s="5">
+        <f>O9-N9</f>
+        <v/>
+      </c>
+      <c r="Q9" s="7">
+        <f>IF(N9=0,"",O9/N9)</f>
+        <v/>
+      </c>
+      <c r="R9" s="5">
+        <f>F9+J9+N9</f>
+        <v/>
+      </c>
+      <c r="S9" s="5">
+        <f>G9+K9+O9</f>
+        <v/>
+      </c>
+      <c r="T9" s="5">
+        <f>S9-R9</f>
+        <v/>
+      </c>
+      <c r="U9" s="7">
+        <f>IF(R9=0,"",S9/R9)</f>
+        <v/>
+      </c>
+      <c r="V9" s="5">
+        <f>B9+R9</f>
+        <v/>
+      </c>
+      <c r="W9" s="5">
+        <f>C9+S9</f>
+        <v/>
+      </c>
+      <c r="X9" s="5">
+        <f>W9-V9</f>
+        <v/>
+      </c>
+      <c r="Y9" s="7">
+        <f>IF(V9=0,"",W9/V9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>أخرى</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>83216589.45</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>193343076.23</v>
+      </c>
+      <c r="D10" s="5">
+        <f>C10-B10</f>
+        <v/>
+      </c>
+      <c r="E10" s="7">
+        <f>IF(B10=0,"",C10/B10)</f>
+        <v/>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>8524595.42</v>
+      </c>
+      <c r="G10" s="5">
+        <f>MAX(7521820.62,35561465.09*'العوامل والدفعات'!D9+'العوامل والدفعات'!B18)</f>
+        <v/>
+      </c>
+      <c r="H10" s="5">
+        <f>G10-F10</f>
+        <v/>
+      </c>
+      <c r="I10" s="7">
+        <f>IF(F10=0,"",G10/F10)</f>
+        <v/>
+      </c>
+      <c r="J10" s="5" t="n">
+        <v>3113156.11</v>
+      </c>
+      <c r="K10" s="5">
+        <f>38749488.20*'العوامل والدفعات'!D9+'العوامل والدفعات'!C18</f>
+        <v/>
+      </c>
+      <c r="L10" s="5">
+        <f>K10-J10</f>
+        <v/>
+      </c>
+      <c r="M10" s="7">
+        <f>IF(J10=0,"",K10/J10)</f>
+        <v/>
+      </c>
+      <c r="N10" s="5" t="n">
+        <v>10370583.68</v>
+      </c>
+      <c r="O10" s="5">
+        <f>35479757.76*'العوامل والدفعات'!D9+'العوامل والدفعات'!D18</f>
+        <v/>
+      </c>
+      <c r="P10" s="5">
+        <f>O10-N10</f>
+        <v/>
+      </c>
+      <c r="Q10" s="7">
+        <f>IF(N10=0,"",O10/N10)</f>
+        <v/>
+      </c>
+      <c r="R10" s="5">
+        <f>F10+J10+N10</f>
+        <v/>
+      </c>
+      <c r="S10" s="5">
+        <f>G10+K10+O10</f>
+        <v/>
+      </c>
+      <c r="T10" s="5">
+        <f>S10-R10</f>
+        <v/>
+      </c>
+      <c r="U10" s="7">
+        <f>IF(R10=0,"",S10/R10)</f>
+        <v/>
+      </c>
+      <c r="V10" s="5">
+        <f>B10+R10</f>
+        <v/>
+      </c>
+      <c r="W10" s="5">
+        <f>C10+S10</f>
+        <v/>
+      </c>
+      <c r="X10" s="5">
+        <f>W10-V10</f>
+        <v/>
+      </c>
+      <c r="Y10" s="7">
+        <f>IF(V10=0,"",W10/V10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>الإجمالي</t>
+        </is>
+      </c>
+      <c r="B11" s="9">
+        <f>SUM(B6:B10)</f>
+        <v/>
+      </c>
+      <c r="C11" s="9">
+        <f>SUM(C6:C10)</f>
+        <v/>
+      </c>
+      <c r="D11" s="9">
+        <f>C11-B11</f>
+        <v/>
+      </c>
+      <c r="E11" s="11">
+        <f>IF(B11=0,"",C11/B11)</f>
+        <v/>
+      </c>
+      <c r="F11" s="9">
+        <f>SUM(F6:F10)</f>
+        <v/>
+      </c>
+      <c r="G11" s="9">
+        <f>SUM(G6:G10)</f>
+        <v/>
+      </c>
+      <c r="H11" s="9">
+        <f>G11-F11</f>
+        <v/>
+      </c>
+      <c r="I11" s="11">
+        <f>IF(F11=0,"",G11/F11)</f>
+        <v/>
+      </c>
+      <c r="J11" s="9">
+        <f>SUM(J6:J10)</f>
+        <v/>
+      </c>
+      <c r="K11" s="9">
+        <f>SUM(K6:K10)</f>
+        <v/>
+      </c>
+      <c r="L11" s="9">
+        <f>K11-J11</f>
+        <v/>
+      </c>
+      <c r="M11" s="11">
+        <f>IF(J11=0,"",K11/J11)</f>
+        <v/>
+      </c>
+      <c r="N11" s="9">
+        <f>SUM(N6:N10)</f>
+        <v/>
+      </c>
+      <c r="O11" s="9">
+        <f>SUM(O6:O10)</f>
+        <v/>
+      </c>
+      <c r="P11" s="9">
+        <f>O11-N11</f>
+        <v/>
+      </c>
+      <c r="Q11" s="11">
+        <f>IF(N11=0,"",O11/N11)</f>
+        <v/>
+      </c>
+      <c r="R11" s="9">
+        <f>SUM(R6:R10)</f>
+        <v/>
+      </c>
+      <c r="S11" s="9">
+        <f>SUM(S6:S10)</f>
+        <v/>
+      </c>
+      <c r="T11" s="9">
+        <f>S11-R11</f>
+        <v/>
+      </c>
+      <c r="U11" s="11">
+        <f>IF(R11=0,"",S11/R11)</f>
+        <v/>
+      </c>
+      <c r="V11" s="9">
+        <f>SUM(V6:V10)</f>
+        <v/>
+      </c>
+      <c r="W11" s="9">
+        <f>SUM(W6:W10)</f>
+        <v/>
+      </c>
+      <c r="X11" s="9">
+        <f>W11-V11</f>
+        <v/>
+      </c>
+      <c r="Y11" s="11">
+        <f>IF(V11=0,"",W11/V11)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="R4:U4"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A2:X2"/>
+    <mergeCell ref="F4:I4"/>
+    <mergeCell ref="V4:Y4"/>
+    <mergeCell ref="J4:M4"/>
+    <mergeCell ref="N4:Q4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Y11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="13" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="13" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="25" max="25"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>الأسوأ: إقفال 2026 بنموذج هولت-وينترز الهجين حسب التبويب (بدون الضريبة)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="44" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>الأسوأ = الحد الأدنى لنطاق ثقة 80% لنموذج هولت-وينترز، بدون عوامل خارجية وبدون الدفعات الاستثنائية (أي لا تصل دفعة تأجير المرافق)، وأكتوبر لا يقل عن المحصل حتى تاريخه.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>التبويب</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>التراكمي يناير–سبتمبر (فعلي)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n"/>
+      <c r="D4" s="3" t="n"/>
+      <c r="E4" s="3" t="n"/>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>أكتوبر</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="n"/>
+      <c r="H4" s="3" t="n"/>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>نوفمبر</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="n"/>
+      <c r="L4" s="3" t="n"/>
+      <c r="M4" s="3" t="n"/>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>ديسمبر</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="n"/>
+      <c r="P4" s="3" t="n"/>
+      <c r="Q4" s="3" t="n"/>
+      <c r="R4" s="3" t="inlineStr">
+        <is>
+          <t>أكتوبر–ديسمبر</t>
+        </is>
+      </c>
+      <c r="S4" s="3" t="n"/>
+      <c r="T4" s="3" t="n"/>
+      <c r="U4" s="3" t="n"/>
+      <c r="V4" s="3" t="inlineStr">
+        <is>
+          <t>إجمالي السنة 2026</t>
+        </is>
+      </c>
+      <c r="W4" s="3" t="n"/>
+      <c r="X4" s="3" t="n"/>
+      <c r="Y4" s="3" t="n"/>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>المستهدف</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>المحصل / المتوقع</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>الفرق عن المستهدف</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>% من المستهدف</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>المستهدف</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>المحصل / المتوقع</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>الفرق عن المستهدف</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>% من المستهدف</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>المستهدف</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>المحصل / المتوقع</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>الفرق عن المستهدف</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>% من المستهدف</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>المستهدف</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="inlineStr">
+        <is>
+          <t>المحصل / المتوقع</t>
+        </is>
+      </c>
+      <c r="P5" s="3" t="inlineStr">
+        <is>
+          <t>الفرق عن المستهدف</t>
+        </is>
+      </c>
+      <c r="Q5" s="3" t="inlineStr">
+        <is>
+          <t>% من المستهدف</t>
+        </is>
+      </c>
+      <c r="R5" s="3" t="inlineStr">
+        <is>
+          <t>المستهدف</t>
+        </is>
+      </c>
+      <c r="S5" s="3" t="inlineStr">
+        <is>
+          <t>المحصل / المتوقع</t>
+        </is>
+      </c>
+      <c r="T5" s="3" t="inlineStr">
+        <is>
+          <t>الفرق عن المستهدف</t>
+        </is>
+      </c>
+      <c r="U5" s="3" t="inlineStr">
+        <is>
+          <t>% من المستهدف</t>
+        </is>
+      </c>
+      <c r="V5" s="3" t="inlineStr">
+        <is>
+          <t>المستهدف</t>
+        </is>
+      </c>
+      <c r="W5" s="3" t="inlineStr">
+        <is>
+          <t>المحصل / المتوقع</t>
+        </is>
+      </c>
+      <c r="X5" s="3" t="inlineStr">
+        <is>
+          <t>الفرق عن المستهدف</t>
+        </is>
+      </c>
+      <c r="Y5" s="3" t="inlineStr">
+        <is>
+          <t>% من المستهدف</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>1038815836.09</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>1052146902.93</v>
+      </c>
+      <c r="D6" s="5">
+        <f>C6-B6</f>
+        <v/>
+      </c>
+      <c r="E6" s="7">
+        <f>IF(B6=0,"",C6/B6)</f>
+        <v/>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>229687321.85</v>
+      </c>
+      <c r="G6" s="5">
+        <f>MAX(33361604.91,76159658.46)</f>
+        <v/>
+      </c>
+      <c r="H6" s="5">
+        <f>G6-F6</f>
+        <v/>
+      </c>
+      <c r="I6" s="7">
+        <f>IF(F6=0,"",G6/F6)</f>
+        <v/>
+      </c>
+      <c r="J6" s="5" t="n">
+        <v>495549226.08</v>
+      </c>
+      <c r="K6" s="5">
+        <f>79165824.83</f>
+        <v/>
+      </c>
+      <c r="L6" s="5">
+        <f>K6-J6</f>
+        <v/>
+      </c>
+      <c r="M6" s="7">
+        <f>IF(J6=0,"",K6/J6)</f>
+        <v/>
+      </c>
+      <c r="N6" s="5" t="n">
+        <v>63384343.05999999</v>
+      </c>
+      <c r="O6" s="5">
+        <f>45928427.08</f>
+        <v/>
+      </c>
+      <c r="P6" s="5">
+        <f>O6-N6</f>
+        <v/>
+      </c>
+      <c r="Q6" s="7">
+        <f>IF(N6=0,"",O6/N6)</f>
+        <v/>
+      </c>
+      <c r="R6" s="5">
+        <f>F6+J6+N6</f>
+        <v/>
+      </c>
+      <c r="S6" s="5">
+        <f>G6+K6+O6</f>
+        <v/>
+      </c>
+      <c r="T6" s="5">
+        <f>S6-R6</f>
+        <v/>
+      </c>
+      <c r="U6" s="7">
+        <f>IF(R6=0,"",S6/R6)</f>
+        <v/>
+      </c>
+      <c r="V6" s="5">
+        <f>B6+R6</f>
+        <v/>
+      </c>
+      <c r="W6" s="5">
+        <f>C6+S6</f>
+        <v/>
+      </c>
+      <c r="X6" s="5">
+        <f>W6-V6</f>
+        <v/>
+      </c>
+      <c r="Y6" s="7">
+        <f>IF(V6=0,"",W6/V6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>895660932.61</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>893640140.0200001</v>
+      </c>
+      <c r="D7" s="5">
+        <f>C7-B7</f>
+        <v/>
+      </c>
+      <c r="E7" s="7">
+        <f>IF(B7=0,"",C7/B7)</f>
+        <v/>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>96839259.07000001</v>
+      </c>
+      <c r="G7" s="5">
+        <f>MAX(47001537.91,80711838.79)</f>
+        <v/>
+      </c>
+      <c r="H7" s="5">
+        <f>G7-F7</f>
+        <v/>
+      </c>
+      <c r="I7" s="7">
+        <f>IF(F7=0,"",G7/F7)</f>
+        <v/>
+      </c>
+      <c r="J7" s="5" t="n">
+        <v>73087705.87</v>
+      </c>
+      <c r="K7" s="5">
+        <f>71282996.57</f>
+        <v/>
+      </c>
+      <c r="L7" s="5">
+        <f>K7-J7</f>
+        <v/>
+      </c>
+      <c r="M7" s="7">
+        <f>IF(J7=0,"",K7/J7)</f>
+        <v/>
+      </c>
+      <c r="N7" s="5" t="n">
+        <v>91097976.65000002</v>
+      </c>
+      <c r="O7" s="5">
+        <f>98039567.38</f>
+        <v/>
+      </c>
+      <c r="P7" s="5">
+        <f>O7-N7</f>
+        <v/>
+      </c>
+      <c r="Q7" s="7">
+        <f>IF(N7=0,"",O7/N7)</f>
+        <v/>
+      </c>
+      <c r="R7" s="5">
+        <f>F7+J7+N7</f>
+        <v/>
+      </c>
+      <c r="S7" s="5">
+        <f>G7+K7+O7</f>
+        <v/>
+      </c>
+      <c r="T7" s="5">
+        <f>S7-R7</f>
+        <v/>
+      </c>
+      <c r="U7" s="7">
+        <f>IF(R7=0,"",S7/R7)</f>
+        <v/>
+      </c>
+      <c r="V7" s="5">
+        <f>B7+R7</f>
+        <v/>
+      </c>
+      <c r="W7" s="5">
+        <f>C7+S7</f>
+        <v/>
+      </c>
+      <c r="X7" s="5">
+        <f>W7-V7</f>
+        <v/>
+      </c>
+      <c r="Y7" s="7">
+        <f>IF(V7=0,"",W7/V7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>جزاءات وغرامات</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>426733084.54</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>638994901.72</v>
+      </c>
+      <c r="D8" s="5">
+        <f>C8-B8</f>
+        <v/>
+      </c>
+      <c r="E8" s="7">
+        <f>IF(B8=0,"",C8/B8)</f>
+        <v/>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>50463196.19</v>
+      </c>
+      <c r="G8" s="5">
+        <f>MAX(33304429.00,21773724.76)</f>
+        <v/>
+      </c>
+      <c r="H8" s="5">
+        <f>G8-F8</f>
+        <v/>
+      </c>
+      <c r="I8" s="7">
+        <f>IF(F8=0,"",G8/F8)</f>
+        <v/>
+      </c>
+      <c r="J8" s="5" t="n">
+        <v>39418777.06</v>
+      </c>
+      <c r="K8" s="5">
+        <f>20861660.82</f>
+        <v/>
+      </c>
+      <c r="L8" s="5">
+        <f>K8-J8</f>
+        <v/>
+      </c>
+      <c r="M8" s="7">
+        <f>IF(J8=0,"",K8/J8)</f>
+        <v/>
+      </c>
+      <c r="N8" s="5" t="n">
+        <v>44888053.81</v>
+      </c>
+      <c r="O8" s="5">
+        <f>26967257.04</f>
+        <v/>
+      </c>
+      <c r="P8" s="5">
+        <f>O8-N8</f>
+        <v/>
+      </c>
+      <c r="Q8" s="7">
+        <f>IF(N8=0,"",O8/N8)</f>
+        <v/>
+      </c>
+      <c r="R8" s="5">
+        <f>F8+J8+N8</f>
+        <v/>
+      </c>
+      <c r="S8" s="5">
+        <f>G8+K8+O8</f>
+        <v/>
+      </c>
+      <c r="T8" s="5">
+        <f>S8-R8</f>
+        <v/>
+      </c>
+      <c r="U8" s="7">
+        <f>IF(R8=0,"",S8/R8)</f>
+        <v/>
+      </c>
+      <c r="V8" s="5">
+        <f>B8+R8</f>
+        <v/>
+      </c>
+      <c r="W8" s="5">
+        <f>C8+S8</f>
+        <v/>
+      </c>
+      <c r="X8" s="5">
+        <f>W8-V8</f>
+        <v/>
+      </c>
+      <c r="Y8" s="7">
+        <f>IF(V8=0,"",W8/V8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>التبغ والإيواء</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>308355656.8</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>209094919.82</v>
+      </c>
+      <c r="D9" s="5">
+        <f>C9-B9</f>
+        <v/>
+      </c>
+      <c r="E9" s="7">
+        <f>IF(B9=0,"",C9/B9)</f>
+        <v/>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>34427181.46</v>
+      </c>
+      <c r="G9" s="5">
+        <f>MAX(17460981.18,19696766.94)</f>
+        <v/>
+      </c>
+      <c r="H9" s="5">
+        <f>G9-F9</f>
+        <v/>
+      </c>
+      <c r="I9" s="7">
+        <f>IF(F9=0,"",G9/F9)</f>
+        <v/>
+      </c>
+      <c r="J9" s="5" t="n">
+        <v>26865316.43</v>
+      </c>
+      <c r="K9" s="5">
+        <f>23378240.43</f>
+        <v/>
+      </c>
+      <c r="L9" s="5">
+        <f>K9-J9</f>
+        <v/>
+      </c>
+      <c r="M9" s="7">
+        <f>IF(J9=0,"",K9/J9)</f>
+        <v/>
+      </c>
+      <c r="N9" s="5" t="n">
+        <v>29501207.8</v>
+      </c>
+      <c r="O9" s="5">
+        <f>21422018.29</f>
+        <v/>
+      </c>
+      <c r="P9" s="5">
+        <f>O9-N9</f>
+        <v/>
+      </c>
+      <c r="Q9" s="7">
+        <f>IF(N9=0,"",O9/N9)</f>
+        <v/>
+      </c>
+      <c r="R9" s="5">
+        <f>F9+J9+N9</f>
+        <v/>
+      </c>
+      <c r="S9" s="5">
+        <f>G9+K9+O9</f>
+        <v/>
+      </c>
+      <c r="T9" s="5">
+        <f>S9-R9</f>
+        <v/>
+      </c>
+      <c r="U9" s="7">
+        <f>IF(R9=0,"",S9/R9)</f>
+        <v/>
+      </c>
+      <c r="V9" s="5">
+        <f>B9+R9</f>
+        <v/>
+      </c>
+      <c r="W9" s="5">
+        <f>C9+S9</f>
+        <v/>
+      </c>
+      <c r="X9" s="5">
+        <f>W9-V9</f>
+        <v/>
+      </c>
+      <c r="Y9" s="7">
+        <f>IF(V9=0,"",W9/V9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>أخرى</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>83216589.45</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>193343076.23</v>
+      </c>
+      <c r="D10" s="5">
+        <f>C10-B10</f>
+        <v/>
+      </c>
+      <c r="E10" s="7">
+        <f>IF(B10=0,"",C10/B10)</f>
+        <v/>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>8524595.42</v>
+      </c>
+      <c r="G10" s="5">
+        <f>MAX(7521820.62,22134264.14)</f>
+        <v/>
+      </c>
+      <c r="H10" s="5">
+        <f>G10-F10</f>
+        <v/>
+      </c>
+      <c r="I10" s="7">
+        <f>IF(F10=0,"",G10/F10)</f>
+        <v/>
+      </c>
+      <c r="J10" s="5" t="n">
+        <v>3113156.11</v>
+      </c>
+      <c r="K10" s="5">
+        <f>24184163.63</f>
+        <v/>
+      </c>
+      <c r="L10" s="5">
+        <f>K10-J10</f>
+        <v/>
+      </c>
+      <c r="M10" s="7">
+        <f>IF(J10=0,"",K10/J10)</f>
+        <v/>
+      </c>
+      <c r="N10" s="5" t="n">
+        <v>10370583.68</v>
+      </c>
+      <c r="O10" s="5">
+        <f>20813077.42</f>
+        <v/>
+      </c>
+      <c r="P10" s="5">
+        <f>O10-N10</f>
+        <v/>
+      </c>
+      <c r="Q10" s="7">
+        <f>IF(N10=0,"",O10/N10)</f>
+        <v/>
+      </c>
+      <c r="R10" s="5">
+        <f>F10+J10+N10</f>
+        <v/>
+      </c>
+      <c r="S10" s="5">
+        <f>G10+K10+O10</f>
+        <v/>
+      </c>
+      <c r="T10" s="5">
+        <f>S10-R10</f>
+        <v/>
+      </c>
+      <c r="U10" s="7">
+        <f>IF(R10=0,"",S10/R10)</f>
+        <v/>
+      </c>
+      <c r="V10" s="5">
+        <f>B10+R10</f>
+        <v/>
+      </c>
+      <c r="W10" s="5">
+        <f>C10+S10</f>
+        <v/>
+      </c>
+      <c r="X10" s="5">
+        <f>W10-V10</f>
+        <v/>
+      </c>
+      <c r="Y10" s="7">
+        <f>IF(V10=0,"",W10/V10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>الإجمالي</t>
+        </is>
+      </c>
+      <c r="B11" s="9">
+        <f>SUM(B6:B10)</f>
+        <v/>
+      </c>
+      <c r="C11" s="9">
+        <f>SUM(C6:C10)</f>
+        <v/>
+      </c>
+      <c r="D11" s="9">
+        <f>C11-B11</f>
+        <v/>
+      </c>
+      <c r="E11" s="11">
+        <f>IF(B11=0,"",C11/B11)</f>
+        <v/>
+      </c>
+      <c r="F11" s="9">
+        <f>SUM(F6:F10)</f>
+        <v/>
+      </c>
+      <c r="G11" s="9">
+        <f>SUM(G6:G10)</f>
+        <v/>
+      </c>
+      <c r="H11" s="9">
+        <f>G11-F11</f>
+        <v/>
+      </c>
+      <c r="I11" s="11">
+        <f>IF(F11=0,"",G11/F11)</f>
+        <v/>
+      </c>
+      <c r="J11" s="9">
+        <f>SUM(J6:J10)</f>
+        <v/>
+      </c>
+      <c r="K11" s="9">
+        <f>SUM(K6:K10)</f>
+        <v/>
+      </c>
+      <c r="L11" s="9">
+        <f>K11-J11</f>
+        <v/>
+      </c>
+      <c r="M11" s="11">
+        <f>IF(J11=0,"",K11/J11)</f>
+        <v/>
+      </c>
+      <c r="N11" s="9">
+        <f>SUM(N6:N10)</f>
+        <v/>
+      </c>
+      <c r="O11" s="9">
+        <f>SUM(O6:O10)</f>
+        <v/>
+      </c>
+      <c r="P11" s="9">
+        <f>O11-N11</f>
+        <v/>
+      </c>
+      <c r="Q11" s="11">
+        <f>IF(N11=0,"",O11/N11)</f>
+        <v/>
+      </c>
+      <c r="R11" s="9">
+        <f>SUM(R6:R10)</f>
+        <v/>
+      </c>
+      <c r="S11" s="9">
+        <f>SUM(S6:S10)</f>
+        <v/>
+      </c>
+      <c r="T11" s="9">
+        <f>S11-R11</f>
+        <v/>
+      </c>
+      <c r="U11" s="11">
+        <f>IF(R11=0,"",S11/R11)</f>
+        <v/>
+      </c>
+      <c r="V11" s="9">
+        <f>SUM(V6:V10)</f>
+        <v/>
+      </c>
+      <c r="W11" s="9">
+        <f>SUM(W6:W10)</f>
+        <v/>
+      </c>
+      <c r="X11" s="9">
+        <f>W11-V11</f>
+        <v/>
+      </c>
+      <c r="Y11" s="11">
+        <f>IF(V11=0,"",W11/V11)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="R4:U4"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A2:X2"/>
+    <mergeCell ref="F4:I4"/>
+    <mergeCell ref="V4:Y4"/>
+    <mergeCell ref="J4:M4"/>
+    <mergeCell ref="N4:Q4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1325,7 +2999,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1702,7 +3376,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>